<commit_message>
update output file generation
</commit_message>
<xml_diff>
--- a/data_out/country_spreadsheets/Albania.xlsx
+++ b/data_out/country_spreadsheets/Albania.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W13"/>
+  <dimension ref="A1:AN13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,87 +461,172 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Median drought days per year</t>
+          <t>Median drought-warning-days</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Maximum recorded drought days per year</t>
+          <t>Maximum recorded drought-warning-days</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>most severe drought year</t>
+          <t>Year of maximum drought-warning-days</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Drought days 2012</t>
+          <t>Warning days 2012</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Drought days 2013</t>
+          <t>Warning days 2013</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Drought days 2014</t>
+          <t>Warning days 2014</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Drought days 2015</t>
+          <t>Warning days 2015</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Drought days 2016</t>
+          <t>Warning days 2016</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>Drought days 2017</t>
+          <t>Warning days 2017</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>Drought days 2018</t>
+          <t>Warning days 2018</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>Drought days 2019</t>
+          <t>Warning days 2019</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>Drought days 2020</t>
+          <t>Warning days 2020</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>Drought days 2021</t>
+          <t>Warning days 2021</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>Drought days 2022</t>
+          <t>Warning days 2022</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>Drought days 2023</t>
+          <t>Warning days 2023</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>Drought days 2024</t>
+          <t>Warning days 2024</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>Drought days 2025</t>
+          <t>Warning days 2025</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Median drought-alert-days</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Maximum recorded drought-alert-days</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>Year of maximum drought-alert-days</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>Alert days 2012</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>Alert days 2013</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>Alert days 2014</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>Alert days 2015</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>Alert days 2016</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>Alert days 2017</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>Alert days 2018</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>Alert days 2019</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>Alert days 2020</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>Alert days 2021</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>Alert days 2022</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>Alert days 2023</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>Alert days 2024</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>Alert days 2025</t>
         </is>
       </c>
     </row>
@@ -621,6 +706,57 @@
       <c r="W2" t="n">
         <v>59.34</v>
       </c>
+      <c r="X2" t="n">
+        <v>11.69</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>58.02</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>2012</v>
+      </c>
+      <c r="AA2" t="n">
+        <v>119.96</v>
+      </c>
+      <c r="AB2" t="n">
+        <v>20.57</v>
+      </c>
+      <c r="AC2" t="n">
+        <v>117.09</v>
+      </c>
+      <c r="AD2" t="n">
+        <v>229.73</v>
+      </c>
+      <c r="AE2" t="n">
+        <v>109.32</v>
+      </c>
+      <c r="AF2" t="n">
+        <v>248.16</v>
+      </c>
+      <c r="AG2" t="n">
+        <v>91.83</v>
+      </c>
+      <c r="AH2" t="n">
+        <v>240.67</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>244.35</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>58.72</v>
+      </c>
+      <c r="AK2" t="n">
+        <v>163.36</v>
+      </c>
+      <c r="AL2" t="n">
+        <v>64.73</v>
+      </c>
+      <c r="AM2" t="n">
+        <v>78.48</v>
+      </c>
+      <c r="AN2" t="n">
+        <v>59.34</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -698,6 +834,57 @@
       <c r="W3" t="n">
         <v>182.02</v>
       </c>
+      <c r="X3" t="n">
+        <v>11.76</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>62.81</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>2012</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>173.45</v>
+      </c>
+      <c r="AB3" t="n">
+        <v>36.3</v>
+      </c>
+      <c r="AC3" t="n">
+        <v>78.47</v>
+      </c>
+      <c r="AD3" t="n">
+        <v>194.26</v>
+      </c>
+      <c r="AE3" t="n">
+        <v>84.39</v>
+      </c>
+      <c r="AF3" t="n">
+        <v>269.56</v>
+      </c>
+      <c r="AG3" t="n">
+        <v>99.90000000000001</v>
+      </c>
+      <c r="AH3" t="n">
+        <v>142.82</v>
+      </c>
+      <c r="AI3" t="n">
+        <v>225.73</v>
+      </c>
+      <c r="AJ3" t="n">
+        <v>132.21</v>
+      </c>
+      <c r="AK3" t="n">
+        <v>159.03</v>
+      </c>
+      <c r="AL3" t="n">
+        <v>147.55</v>
+      </c>
+      <c r="AM3" t="n">
+        <v>192.85</v>
+      </c>
+      <c r="AN3" t="n">
+        <v>182.02</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -775,6 +962,57 @@
       <c r="W4" t="n">
         <v>168.36</v>
       </c>
+      <c r="X4" t="n">
+        <v>9.33</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>72.58</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>2012</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>179.35</v>
+      </c>
+      <c r="AB4" t="n">
+        <v>30.45</v>
+      </c>
+      <c r="AC4" t="n">
+        <v>30.71</v>
+      </c>
+      <c r="AD4" t="n">
+        <v>113.82</v>
+      </c>
+      <c r="AE4" t="n">
+        <v>16.91</v>
+      </c>
+      <c r="AF4" t="n">
+        <v>192.95</v>
+      </c>
+      <c r="AG4" t="n">
+        <v>106.87</v>
+      </c>
+      <c r="AH4" t="n">
+        <v>76.04000000000001</v>
+      </c>
+      <c r="AI4" t="n">
+        <v>94.38</v>
+      </c>
+      <c r="AJ4" t="n">
+        <v>149.87</v>
+      </c>
+      <c r="AK4" t="n">
+        <v>130.75</v>
+      </c>
+      <c r="AL4" t="n">
+        <v>55.24</v>
+      </c>
+      <c r="AM4" t="n">
+        <v>141.48</v>
+      </c>
+      <c r="AN4" t="n">
+        <v>168.36</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -852,6 +1090,57 @@
       <c r="W5" t="n">
         <v>123.21</v>
       </c>
+      <c r="X5" t="n">
+        <v>13.18</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>49.57</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>2012</v>
+      </c>
+      <c r="AA5" t="n">
+        <v>153.37</v>
+      </c>
+      <c r="AB5" t="n">
+        <v>17.83</v>
+      </c>
+      <c r="AC5" t="n">
+        <v>58.84</v>
+      </c>
+      <c r="AD5" t="n">
+        <v>239.78</v>
+      </c>
+      <c r="AE5" t="n">
+        <v>84.12</v>
+      </c>
+      <c r="AF5" t="n">
+        <v>266.82</v>
+      </c>
+      <c r="AG5" t="n">
+        <v>112.48</v>
+      </c>
+      <c r="AH5" t="n">
+        <v>154.26</v>
+      </c>
+      <c r="AI5" t="n">
+        <v>219.72</v>
+      </c>
+      <c r="AJ5" t="n">
+        <v>131.05</v>
+      </c>
+      <c r="AK5" t="n">
+        <v>160.74</v>
+      </c>
+      <c r="AL5" t="n">
+        <v>64.59999999999999</v>
+      </c>
+      <c r="AM5" t="n">
+        <v>79.89</v>
+      </c>
+      <c r="AN5" t="n">
+        <v>123.21</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
@@ -929,6 +1218,57 @@
       <c r="W6" t="n">
         <v>129.01</v>
       </c>
+      <c r="X6" t="n">
+        <v>7.87</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>41.31</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>2012</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>135.6</v>
+      </c>
+      <c r="AB6" t="n">
+        <v>18.71</v>
+      </c>
+      <c r="AC6" t="n">
+        <v>13.88</v>
+      </c>
+      <c r="AD6" t="n">
+        <v>217.57</v>
+      </c>
+      <c r="AE6" t="n">
+        <v>49.28</v>
+      </c>
+      <c r="AF6" t="n">
+        <v>235.37</v>
+      </c>
+      <c r="AG6" t="n">
+        <v>119.61</v>
+      </c>
+      <c r="AH6" t="n">
+        <v>82.91</v>
+      </c>
+      <c r="AI6" t="n">
+        <v>148.52</v>
+      </c>
+      <c r="AJ6" t="n">
+        <v>138.12</v>
+      </c>
+      <c r="AK6" t="n">
+        <v>133.89</v>
+      </c>
+      <c r="AL6" t="n">
+        <v>44.23</v>
+      </c>
+      <c r="AM6" t="n">
+        <v>45.16</v>
+      </c>
+      <c r="AN6" t="n">
+        <v>129.01</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
@@ -1006,6 +1346,57 @@
       <c r="W7" t="n">
         <v>120.04</v>
       </c>
+      <c r="X7" t="n">
+        <v>5.77</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>48.23</v>
+      </c>
+      <c r="Z7" t="n">
+        <v>2012</v>
+      </c>
+      <c r="AA7" t="n">
+        <v>228.31</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>12.15</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>55.87</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>30.79</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>6.38</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>194.25</v>
+      </c>
+      <c r="AG7" t="n">
+        <v>82</v>
+      </c>
+      <c r="AH7" t="n">
+        <v>132.23</v>
+      </c>
+      <c r="AI7" t="n">
+        <v>73.53</v>
+      </c>
+      <c r="AJ7" t="n">
+        <v>65.91</v>
+      </c>
+      <c r="AK7" t="n">
+        <v>94.7</v>
+      </c>
+      <c r="AL7" t="n">
+        <v>61.89</v>
+      </c>
+      <c r="AM7" t="n">
+        <v>27.55</v>
+      </c>
+      <c r="AN7" t="n">
+        <v>120.04</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -1083,6 +1474,57 @@
       <c r="W8" t="n">
         <v>157.14</v>
       </c>
+      <c r="X8" t="n">
+        <v>12.13</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>42.41</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>2012</v>
+      </c>
+      <c r="AA8" t="n">
+        <v>219.02</v>
+      </c>
+      <c r="AB8" t="n">
+        <v>64.34999999999999</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>103.83</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>183.75</v>
+      </c>
+      <c r="AE8" t="n">
+        <v>85.88</v>
+      </c>
+      <c r="AF8" t="n">
+        <v>261.3</v>
+      </c>
+      <c r="AG8" t="n">
+        <v>100.29</v>
+      </c>
+      <c r="AH8" t="n">
+        <v>149.35</v>
+      </c>
+      <c r="AI8" t="n">
+        <v>225.97</v>
+      </c>
+      <c r="AJ8" t="n">
+        <v>138.67</v>
+      </c>
+      <c r="AK8" t="n">
+        <v>147.18</v>
+      </c>
+      <c r="AL8" t="n">
+        <v>106.04</v>
+      </c>
+      <c r="AM8" t="n">
+        <v>179.46</v>
+      </c>
+      <c r="AN8" t="n">
+        <v>157.14</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
@@ -1160,6 +1602,57 @@
       <c r="W9" t="n">
         <v>264.06</v>
       </c>
+      <c r="X9" t="n">
+        <v>11.06</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>26.73</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>2012</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>221.59</v>
+      </c>
+      <c r="AB9" t="n">
+        <v>4.13</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>45.52</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>51.14</v>
+      </c>
+      <c r="AE9" t="n">
+        <v>9.75</v>
+      </c>
+      <c r="AF9" t="n">
+        <v>248.22</v>
+      </c>
+      <c r="AG9" t="n">
+        <v>51.74</v>
+      </c>
+      <c r="AH9" t="n">
+        <v>85.51000000000001</v>
+      </c>
+      <c r="AI9" t="n">
+        <v>96</v>
+      </c>
+      <c r="AJ9" t="n">
+        <v>65.01000000000001</v>
+      </c>
+      <c r="AK9" t="n">
+        <v>195.25</v>
+      </c>
+      <c r="AL9" t="n">
+        <v>162.19</v>
+      </c>
+      <c r="AM9" t="n">
+        <v>118.29</v>
+      </c>
+      <c r="AN9" t="n">
+        <v>264.06</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
@@ -1237,6 +1730,57 @@
       <c r="W10" t="n">
         <v>212.07</v>
       </c>
+      <c r="X10" t="n">
+        <v>4.97</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>55.96</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>2012</v>
+      </c>
+      <c r="AA10" t="n">
+        <v>218.67</v>
+      </c>
+      <c r="AB10" t="n">
+        <v>38.67</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>133.93</v>
+      </c>
+      <c r="AD10" t="n">
+        <v>244.04</v>
+      </c>
+      <c r="AE10" t="n">
+        <v>140.19</v>
+      </c>
+      <c r="AF10" t="n">
+        <v>334.84</v>
+      </c>
+      <c r="AG10" t="n">
+        <v>97.01000000000001</v>
+      </c>
+      <c r="AH10" t="n">
+        <v>142.79</v>
+      </c>
+      <c r="AI10" t="n">
+        <v>198.69</v>
+      </c>
+      <c r="AJ10" t="n">
+        <v>67.78</v>
+      </c>
+      <c r="AK10" t="n">
+        <v>228.23</v>
+      </c>
+      <c r="AL10" t="n">
+        <v>201.01</v>
+      </c>
+      <c r="AM10" t="n">
+        <v>230.84</v>
+      </c>
+      <c r="AN10" t="n">
+        <v>212.07</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
@@ -1314,6 +1858,57 @@
       <c r="W11" t="n">
         <v>216.34</v>
       </c>
+      <c r="X11" t="n">
+        <v>7.36</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>35.56</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>2019</v>
+      </c>
+      <c r="AA11" t="n">
+        <v>179.44</v>
+      </c>
+      <c r="AB11" t="n">
+        <v>22.3</v>
+      </c>
+      <c r="AC11" t="n">
+        <v>22.12</v>
+      </c>
+      <c r="AD11" t="n">
+        <v>29.42</v>
+      </c>
+      <c r="AE11" t="n">
+        <v>15.41</v>
+      </c>
+      <c r="AF11" t="n">
+        <v>212</v>
+      </c>
+      <c r="AG11" t="n">
+        <v>71.95</v>
+      </c>
+      <c r="AH11" t="n">
+        <v>177.87</v>
+      </c>
+      <c r="AI11" t="n">
+        <v>171.36</v>
+      </c>
+      <c r="AJ11" t="n">
+        <v>123.74</v>
+      </c>
+      <c r="AK11" t="n">
+        <v>167.68</v>
+      </c>
+      <c r="AL11" t="n">
+        <v>46.78</v>
+      </c>
+      <c r="AM11" t="n">
+        <v>198.57</v>
+      </c>
+      <c r="AN11" t="n">
+        <v>216.34</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="inlineStr">
@@ -1391,6 +1986,57 @@
       <c r="W12" t="n">
         <v>111.68</v>
       </c>
+      <c r="X12" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>22.96</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>2012</v>
+      </c>
+      <c r="AA12" t="n">
+        <v>86.17</v>
+      </c>
+      <c r="AB12" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="AC12" t="n">
+        <v>8.83</v>
+      </c>
+      <c r="AD12" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="AE12" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="AF12" t="n">
+        <v>86.53</v>
+      </c>
+      <c r="AG12" t="n">
+        <v>24.21</v>
+      </c>
+      <c r="AH12" t="n">
+        <v>63.02</v>
+      </c>
+      <c r="AI12" t="n">
+        <v>33.09</v>
+      </c>
+      <c r="AJ12" t="n">
+        <v>37.28</v>
+      </c>
+      <c r="AK12" t="n">
+        <v>63.76</v>
+      </c>
+      <c r="AL12" t="n">
+        <v>16.96</v>
+      </c>
+      <c r="AM12" t="n">
+        <v>39.54</v>
+      </c>
+      <c r="AN12" t="n">
+        <v>111.68</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr">
@@ -1466,6 +2112,57 @@
         <v>232.45</v>
       </c>
       <c r="W13" t="n">
+        <v>191.32</v>
+      </c>
+      <c r="X13" t="n">
+        <v>6.08</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>32.06</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>2022</v>
+      </c>
+      <c r="AA13" t="n">
+        <v>164.16</v>
+      </c>
+      <c r="AB13" t="n">
+        <v>13.04</v>
+      </c>
+      <c r="AC13" t="n">
+        <v>30.94</v>
+      </c>
+      <c r="AD13" t="n">
+        <v>93.14</v>
+      </c>
+      <c r="AE13" t="n">
+        <v>96.68000000000001</v>
+      </c>
+      <c r="AF13" t="n">
+        <v>267.75</v>
+      </c>
+      <c r="AG13" t="n">
+        <v>82.84</v>
+      </c>
+      <c r="AH13" t="n">
+        <v>184.69</v>
+      </c>
+      <c r="AI13" t="n">
+        <v>179.37</v>
+      </c>
+      <c r="AJ13" t="n">
+        <v>55.83</v>
+      </c>
+      <c r="AK13" t="n">
+        <v>188.44</v>
+      </c>
+      <c r="AL13" t="n">
+        <v>159.83</v>
+      </c>
+      <c r="AM13" t="n">
+        <v>232.45</v>
+      </c>
+      <c r="AN13" t="n">
         <v>191.32</v>
       </c>
     </row>

</xml_diff>